<commit_message>
Add Login Test Case and Login Test Data
</commit_message>
<xml_diff>
--- a/04_Test_Case/TestCase_Login.xlsx
+++ b/04_Test_Case/TestCase_Login.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Manual-Tester-Portfolio\04_Test_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{247F0BEE-D7EB-4BB1-A858-788785CE4829}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A82611AF-73F4-48B7-9874-A5680849EA4A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4116" yWindow="1248" windowWidth="17280" windowHeight="8964" xr2:uid="{05835D8B-0112-4498-8A28-0E2D20A4BDFF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05835D8B-0112-4498-8A28-0E2D20A4BDFF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="TestCase Login" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,9 +33,398 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="114">
+  <si>
+    <t>TC ID</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Preconditions</t>
+  </si>
+  <si>
+    <t>Steps</t>
+  </si>
+  <si>
+    <t>Test Data</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_001</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_002</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_003</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_004</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_005</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_006</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_007</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_008</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_009</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_010</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_011</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_012</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_013</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_014</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_015</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_016</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_017</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_018</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_019</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_020</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_021</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_022</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công với Email và Password hợp lệ</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Password nhỏ hơn 8 ký tự</t>
+  </si>
+  <si>
+    <t>Cho phép đăng nhập với Password đúng 20 ký tự</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Password lớn hơn 20 ký tự</t>
+  </si>
+  <si>
+    <t>Password phân biệt chữ hoa và chữ thường</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập khi Password chỉ chứa khoảng trắng</t>
+  </si>
+  <si>
+    <t>Đăng nhập sai 1 lần và hiển thị thông báo lỗi</t>
+  </si>
+  <si>
+    <t>Đăng nhập sai liên tiếp 5 lần nhưng tài khoản chưa bị khóa</t>
+  </si>
+  <si>
+    <t>Tài khoản bị khóa sau lần đăng nhập sai thứ 6</t>
+  </si>
+  <si>
+    <t>Cho phép đăng nhập lại sau khi hết thời gian khóa (15 phút)</t>
+  </si>
+  <si>
+    <t>Hiển thị Password khi nhấn biểu tượng Show Password</t>
+  </si>
+  <si>
+    <t>Ẩn Password khi nhấn lại biểu tượng Show Password</t>
+  </si>
+  <si>
+    <t>Ghi nhớ trạng thái đăng nhập khi chọn Remember Me</t>
+  </si>
+  <si>
+    <t>Không ghi nhớ trạng thái đăng nhập khi không chọn Remember Me</t>
+  </si>
+  <si>
+    <t>Vẫn giữ trạng thái đăng nhập sau khi đóng và mở lại trình duyệt khi đã chọn Remember Me</t>
+  </si>
+  <si>
+    <t>Not run</t>
+  </si>
+  <si>
+    <t>Người dùng có tài khoản hợp lệ và đang ở màn hình Login</t>
+  </si>
+  <si>
+    <t>1. Mở trang Login
+2. Nhập email hợp lệ
+3. Nhập password hợp lệ
+4. Nhấn nút login</t>
+  </si>
+  <si>
+    <t>1. Để trống email
+2. Nhập password hợp lệ
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>Người dùng đang ở màn hình Login</t>
+  </si>
+  <si>
+    <t>1. Nhập email sai định dạng
+2. Nhập password hợp lệ
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập. Hệ thống hiển thị thông báo lỗi theo Requirement.</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập khi để trống Email</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Email sai định dạng</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Email sai định dạng.</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Email chưa được đăng ký</t>
+  </si>
+  <si>
+    <t>1. Nhập email chưa đăng ký
+2. Nhập password bất kỳ
+3. Nhấp Login</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập. Hiển thị thông báo "Email hoặc Password không đúng."</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập khi để trống Password</t>
+  </si>
+  <si>
+    <t>1. Nhập email hợp lệ
+2. Để trống password 
+3. Nhấp Login</t>
+  </si>
+  <si>
+    <t>1. Nhập email hợp lệ
+2. Nhập Password có ít hơn 8 ký tự
+3. Nhấp Login</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Password nhỏ hơn 8 ký tự.</t>
+  </si>
+  <si>
+    <t>Cho phép đăng nhập với Password đúng 8 ký tự (mức tối thiểu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người dùng có tài khoản hợp lệ </t>
+  </si>
+  <si>
+    <t>1. Nhập email hợp lệ
+2. Nhập Password đúng 8 ký tự
+3. Nhấp Login</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công và chuyển đến Dashboard.</t>
+  </si>
+  <si>
+    <t>1. Nhập email hợp lệ
+2. Nhập Password đúng 20 ký tự
+3. Nhấp Login</t>
+  </si>
+  <si>
+    <t>TD001</t>
+  </si>
+  <si>
+    <t>TD002</t>
+  </si>
+  <si>
+    <t>TD009</t>
+  </si>
+  <si>
+    <t>TD010</t>
+  </si>
+  <si>
+    <t>TD011</t>
+  </si>
+  <si>
+    <t>TD012</t>
+  </si>
+  <si>
+    <t>TD005</t>
+  </si>
+  <si>
+    <t>TD006</t>
+  </si>
+  <si>
+    <t>TD008</t>
+  </si>
+  <si>
+    <t>TD003</t>
+  </si>
+  <si>
+    <t>1. Nhập email hợp lệ
+2. Nhập Password hơn 20 ký tự (21 ký tự)
+3. Nhấp Login</t>
+  </si>
+  <si>
+    <t>TD004</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Password lớn hơn 20 ký tự.</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Password không chính xác</t>
+  </si>
+  <si>
+    <t>1. Nhập email 
+2. Nhập password sai
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>TD007</t>
+  </si>
+  <si>
+    <t>1. Nhập email 
+2. Nhập password khác chữ hoa/chữ thường so với mật khẩu đã đăng ký
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>1. Nhập email 
+2. Nhập password chỉ chứa khoảng trắng
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>1. Nhập email 
+2. Nhập password sai
+3. Nhấn login liên tiếp 5 lần</t>
+  </si>
+  <si>
+    <t>1. Nhập email 
+2. Nhập password sai
+3. Nhấn login liên tiếp 6 lần</t>
+  </si>
+  <si>
+    <t>Tài khoản bị khóa trong 15 phút theo Requirement.</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Tài khoản đã bị khóa 15 phút</t>
+  </si>
+  <si>
+    <t>1. Chờ đủ 15 phút
+2. Nhập email đúng
+3. Nhập password đúng
+4. Nhấn login</t>
+  </si>
+  <si>
+    <t>1. Nhập password
+2. Nhấn biểu tượng Show password</t>
+  </si>
+  <si>
+    <t>Password được hiển thị đúng với dữ liệu đã nhập.</t>
+  </si>
+  <si>
+    <t>1. Nhấn lại biểu tượng Show password</t>
+  </si>
+  <si>
+    <t>Password đang được hiển thị</t>
+  </si>
+  <si>
+    <t>Người dùng đã có tài khoản hợp lệ</t>
+  </si>
+  <si>
+    <t>1. Nhập Email và Password hợp lệ
+2. Chọn remember me
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công. Hệ thống ghi nhớ trạng thái đăng nhập theo Requirement.</t>
+  </si>
+  <si>
+    <t>1. Nhập Email và Password hợp lệ
+2. Không chọn remember me
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>Người dùng đã đăng nhập thành công và đã chọn Remember Me</t>
+  </si>
+  <si>
+    <t>1. Đóng trình duyệt
+2. Mở lại trình duyệt
+3. Truy cập hệ thống</t>
+  </si>
+  <si>
+    <t>Người dùng vẫn ở trạng thái đăng nhập</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập khi để trống email và password</t>
+  </si>
+  <si>
+    <t>1. Để trống email 
+2. Để trống password 
+3. Nhấn login</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập. Hiển thị thông báo "Email hoặc Password không đúng.". Tài khoản chưa bị khóa.</t>
+  </si>
+  <si>
+    <t>Sau khi hết thời gian khóa 15 phút, người dùng có thể đăng nhập thành công và chuyển đến Dashboard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Password được ẩn trở lại bằng ký tự che. </t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công.
+Sau khi đóng trình duyệt, người dùng phải đăng nhập lại.</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công và chuyển đến Dashboard. Dashboard hiển thị "Xin chào Nguyễn Văn A".</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -43,16 +432,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,18 +469,128 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF23C317"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF5B5B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFB9B9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF4747"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF4747"/>
+      <color rgb="FFFF5B5B"/>
+      <color rgb="FF23C317"/>
+      <color rgb="FFFFB9B9"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -380,9 +899,766 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD06D675-C1C1-4A3D-B3EE-03E6DB288C74}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.77734375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="19.21875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="40.5546875" customWidth="1"/>
+    <col min="4" max="4" width="35.44140625" customWidth="1"/>
+    <col min="5" max="5" width="55" customWidth="1"/>
+    <col min="6" max="6" width="35.44140625" customWidth="1"/>
+    <col min="7" max="7" width="56.109375" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="16.21875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="4" customFormat="1" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="6"/>
+      <c r="I3" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="6"/>
+      <c r="I4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="6"/>
+      <c r="I12" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="6"/>
+      <c r="I16" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" s="6"/>
+      <c r="I17" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H18" s="6"/>
+      <c r="I18" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H19" s="6"/>
+      <c r="I19" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="H20" s="6"/>
+      <c r="I20" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="H21" s="6"/>
+      <c r="I21" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="6"/>
+      <c r="I22" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H23" s="6"/>
+      <c r="I23" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="J2:J24">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Critical">
+      <formula>NOT(ISERROR(SEARCH("Critical",J2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="Low">
+      <formula>NOT(ISERROR(SEARCH("Low",J2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="Medium">
+      <formula>NOT(ISERROR(SEARCH("Medium",J2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="High">
+      <formula>NOT(ISERROR(SEARCH("High",J2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I24">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Not run">
+      <formula>NOT(ISERROR(SEARCH("Not run",I2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J24" xr:uid="{4F90E516-AFDB-4655-8061-B3B3E4DA67FB}">
+      <formula1>"Critical, High, Medium, Low"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I24" xr:uid="{0D375ED5-87A5-4052-A211-29034E1799F6}">
+      <formula1>"Not run, Pass, Fail"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>